<commit_message>
update timesheet week 4 devi
</commit_message>
<xml_diff>
--- a/DeviMaya_S388017/Timesheet Devi Maya.xlsx
+++ b/DeviMaya_S388017/Timesheet Devi Maya.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\azra\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/devi/Documents/GitHub/PRT585-SOFTWARE-ENGINEERING-PRACTICE/DeviMaya_S388017/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{57728B68-2B6C-4DCE-990E-862230EAD445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E971303-6967-C44D-B05F-FBB149CC50C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Individual timesheet" sheetId="2" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="25">
   <si>
     <t>EACH INDIVIDUAL MUST HAVE TO ENTER 6 HOURS TIME LOGGING IN THIS PAGE PER EACH WEEK</t>
   </si>
@@ -101,13 +101,33 @@
   <si>
     <t>Refreshing Database Fundamentals
 (Using materials from last semester's Database Fundamentals class)</t>
+  </si>
+  <si>
+    <t>Week-4</t>
+  </si>
+  <si>
+    <t>Project work: Refine project scope &amp; functional requirements</t>
+  </si>
+  <si>
+    <t>Project work: define use cases &amp; write use case description</t>
+  </si>
+  <si>
+    <t>Project work: define traceability matrix</t>
+  </si>
+  <si>
+    <t>Project work: prepare work breakdown structures &amp; gantt chart
+Use mermaid gantt chart for now</t>
+  </si>
+  <si>
+    <t>Project work: start drafting ERD
+Current diagram is using PlantUML, will try to move to better visualisation option later</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -175,12 +195,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
     </font>
     <font>
       <u/>
@@ -194,18 +214,19 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -263,7 +284,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -322,6 +343,9 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -342,9 +366,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -382,7 +406,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -488,7 +512,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -630,7 +654,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -639,17 +663,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F177"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" style="4" customWidth="1"/>
-    <col min="2" max="2" width="22.28515625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="36.42578125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" style="4" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="36.5" style="4" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" style="4" customWidth="1"/>
     <col min="5" max="5" width="122" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="4"/>
+    <col min="6" max="16384" width="9.1640625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -659,7 +683,7 @@
       <c r="E1" s="3"/>
       <c r="F1" s="2"/>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -676,7 +700,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15">
+    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -693,7 +717,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15">
+    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="18" t="s">
         <v>6</v>
       </c>
@@ -710,7 +734,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15">
+    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="18" t="s">
         <v>6</v>
       </c>
@@ -727,7 +751,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15">
+    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="18" t="s">
         <v>6</v>
       </c>
@@ -744,7 +768,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15">
+    <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="18" t="s">
         <v>6</v>
       </c>
@@ -761,7 +785,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="30.75">
+    <row r="8" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="18" t="s">
         <v>6</v>
       </c>
@@ -778,496 +802,538 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B9" s="7"/>
     </row>
-    <row r="10" spans="1:6" ht="15"/>
-    <row r="11" spans="1:6" ht="15"/>
-    <row r="12" spans="1:6">
-      <c r="E12" s="4"/>
-    </row>
-    <row r="13" spans="1:6" ht="15"/>
-    <row r="14" spans="1:6" ht="15"/>
-    <row r="15" spans="1:6" ht="15"/>
-    <row r="16" spans="1:6" ht="15"/>
-    <row r="17" spans="5:5" ht="15"/>
-    <row r="18" spans="5:5" ht="15"/>
-    <row r="19" spans="5:5" ht="15">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="4">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="4">
+        <v>2</v>
+      </c>
+      <c r="E11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="25" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E19" s="19"/>
     </row>
-    <row r="20" spans="5:5" ht="15"/>
-    <row r="21" spans="5:5" ht="15"/>
-    <row r="22" spans="5:5" ht="15"/>
-    <row r="23" spans="5:5" ht="15"/>
-    <row r="24" spans="5:5" ht="15"/>
-    <row r="25" spans="5:5" ht="15"/>
-    <row r="26" spans="5:5" ht="15"/>
-    <row r="27" spans="5:5" ht="15"/>
-    <row r="28" spans="5:5" ht="15"/>
-    <row r="29" spans="5:5" ht="15"/>
-    <row r="30" spans="5:5" ht="15"/>
-    <row r="31" spans="5:5" ht="15"/>
-    <row r="32" spans="5:5" ht="15"/>
-    <row r="33" spans="5:5" ht="15"/>
-    <row r="34" spans="5:5" ht="15"/>
-    <row r="35" spans="5:5" ht="15"/>
-    <row r="36" spans="5:5">
+    <row r="36" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E36"/>
     </row>
-    <row r="37" spans="5:5">
+    <row r="37" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E37"/>
     </row>
-    <row r="38" spans="5:5">
+    <row r="38" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E38"/>
     </row>
-    <row r="39" spans="5:5">
+    <row r="39" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E39"/>
     </row>
-    <row r="40" spans="5:5">
+    <row r="40" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E40"/>
     </row>
-    <row r="41" spans="5:5">
+    <row r="41" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E41" s="24"/>
     </row>
-    <row r="42" spans="5:5">
+    <row r="42" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E42" s="24"/>
     </row>
-    <row r="43" spans="5:5">
+    <row r="43" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E43" s="24"/>
     </row>
-    <row r="44" spans="5:5">
+    <row r="44" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E44" s="24"/>
     </row>
-    <row r="45" spans="5:5">
+    <row r="45" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E45" s="24"/>
     </row>
-    <row r="46" spans="5:5">
+    <row r="46" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E46" s="24"/>
     </row>
-    <row r="47" spans="5:5" ht="15"/>
-    <row r="48" spans="5:5" ht="15">
+    <row r="48" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E48" s="9"/>
     </row>
-    <row r="49" spans="4:5" ht="15">
+    <row r="49" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D49" s="10"/>
       <c r="E49" s="9"/>
     </row>
-    <row r="50" spans="4:5" ht="15"/>
-    <row r="51" spans="4:5" ht="15"/>
-    <row r="52" spans="4:5" ht="15"/>
-    <row r="53" spans="4:5" ht="15"/>
-    <row r="54" spans="4:5" ht="15"/>
-    <row r="55" spans="4:5" ht="15"/>
-    <row r="56" spans="4:5" ht="15"/>
-    <row r="57" spans="4:5" ht="15"/>
-    <row r="58" spans="4:5" ht="15"/>
-    <row r="59" spans="4:5" ht="15"/>
-    <row r="60" spans="4:5" ht="15"/>
-    <row r="61" spans="4:5" ht="15"/>
-    <row r="62" spans="4:5" ht="15"/>
-    <row r="63" spans="4:5" ht="15"/>
-    <row r="64" spans="4:5" ht="15"/>
-    <row r="65" spans="1:5" ht="15"/>
-    <row r="66" spans="1:5">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E66" s="4"/>
     </row>
-    <row r="67" spans="1:5" ht="15"/>
-    <row r="68" spans="1:5" ht="77.25" customHeight="1"/>
-    <row r="69" spans="1:5" ht="73.5" customHeight="1"/>
-    <row r="70" spans="1:5" ht="15"/>
-    <row r="71" spans="1:5" ht="15"/>
-    <row r="72" spans="1:5" ht="15"/>
-    <row r="73" spans="1:5" ht="15"/>
-    <row r="74" spans="1:5" ht="15">
+    <row r="68" spans="1:5" ht="77.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="69" spans="1:5" ht="73.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" s="11"/>
       <c r="B74" s="11"/>
       <c r="C74" s="11"/>
     </row>
-    <row r="75" spans="1:5" ht="15">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" s="11"/>
       <c r="B75" s="11"/>
       <c r="C75" s="11"/>
     </row>
-    <row r="76" spans="1:5" ht="15">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" s="11"/>
       <c r="B76" s="11"/>
       <c r="C76" s="11"/>
     </row>
-    <row r="77" spans="1:5" ht="15">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" s="11"/>
       <c r="B77" s="11"/>
       <c r="C77" s="11"/>
     </row>
-    <row r="78" spans="1:5" ht="15">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" s="11"/>
       <c r="B78" s="11"/>
       <c r="C78" s="11"/>
     </row>
-    <row r="79" spans="1:5" ht="15">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" s="11"/>
     </row>
-    <row r="80" spans="1:5" ht="15">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" s="18"/>
     </row>
-    <row r="81" spans="1:5" ht="15">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" s="18"/>
     </row>
-    <row r="82" spans="1:5">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" s="18"/>
       <c r="E82" s="12"/>
     </row>
-    <row r="83" spans="1:5" ht="15">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" s="18"/>
     </row>
-    <row r="84" spans="1:5" ht="15">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84" s="18"/>
     </row>
-    <row r="85" spans="1:5" ht="15">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B85"/>
     </row>
-    <row r="86" spans="1:5" ht="15">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B86"/>
     </row>
-    <row r="87" spans="1:5">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B87"/>
       <c r="E87"/>
     </row>
-    <row r="88" spans="1:5" ht="15">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B88"/>
     </row>
-    <row r="89" spans="1:5" ht="15">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B89"/>
     </row>
-    <row r="90" spans="1:5">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B90"/>
       <c r="E90"/>
     </row>
-    <row r="91" spans="1:5" ht="15"/>
-    <row r="92" spans="1:5" ht="15"/>
-    <row r="93" spans="1:5" ht="15">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" s="13"/>
       <c r="B93" s="13"/>
       <c r="C93" s="13"/>
       <c r="D93" s="13"/>
       <c r="E93" s="14"/>
     </row>
-    <row r="94" spans="1:5" ht="15">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" s="13"/>
       <c r="B94" s="13"/>
       <c r="C94" s="13"/>
       <c r="D94" s="13"/>
       <c r="E94" s="14"/>
     </row>
-    <row r="95" spans="1:5" ht="15">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95" s="13"/>
       <c r="B95" s="13"/>
       <c r="C95" s="13"/>
       <c r="D95" s="13"/>
       <c r="E95" s="14"/>
     </row>
-    <row r="96" spans="1:5" ht="18.75" customHeight="1">
+    <row r="96" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="13"/>
       <c r="B96" s="13"/>
       <c r="C96" s="13"/>
       <c r="D96" s="13"/>
       <c r="E96" s="14"/>
     </row>
-    <row r="97" spans="1:5" ht="15">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97" s="13"/>
       <c r="B97" s="13"/>
       <c r="C97" s="13"/>
       <c r="D97" s="13"/>
       <c r="E97" s="14"/>
     </row>
-    <row r="98" spans="1:5" ht="15">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98" s="13"/>
       <c r="B98" s="13"/>
       <c r="C98" s="13"/>
       <c r="D98" s="13"/>
       <c r="E98" s="14"/>
     </row>
-    <row r="99" spans="1:5" ht="15"/>
-    <row r="100" spans="1:5" ht="15"/>
-    <row r="101" spans="1:5">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101" s="13"/>
       <c r="E101"/>
     </row>
-    <row r="102" spans="1:5">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102" s="13"/>
       <c r="E102"/>
     </row>
-    <row r="103" spans="1:5">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103" s="13"/>
       <c r="E103"/>
     </row>
-    <row r="104" spans="1:5">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" s="13"/>
       <c r="E104"/>
     </row>
-    <row r="105" spans="1:5">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105" s="13"/>
       <c r="E105"/>
     </row>
-    <row r="106" spans="1:5">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" s="13"/>
       <c r="E106"/>
     </row>
-    <row r="107" spans="1:5" ht="15"/>
-    <row r="108" spans="1:5" ht="15">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108" s="13"/>
     </row>
-    <row r="109" spans="1:5">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109" s="13"/>
       <c r="B109"/>
       <c r="E109" s="4"/>
     </row>
-    <row r="110" spans="1:5" ht="15">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110" s="13"/>
     </row>
-    <row r="111" spans="1:5">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111" s="13"/>
       <c r="E111"/>
     </row>
-    <row r="112" spans="1:5" ht="15">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A112" s="13"/>
     </row>
-    <row r="113" spans="1:5" ht="15">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A113" s="13"/>
     </row>
-    <row r="114" spans="1:5" ht="15"/>
-    <row r="115" spans="1:5" ht="15">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A115" s="13"/>
       <c r="D115" s="15"/>
     </row>
-    <row r="116" spans="1:5" ht="15">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116" s="13"/>
       <c r="D116" s="15"/>
     </row>
-    <row r="117" spans="1:5" ht="15">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117" s="13"/>
       <c r="D117" s="15"/>
     </row>
-    <row r="118" spans="1:5" ht="35.25" customHeight="1">
+    <row r="118" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="13"/>
       <c r="D118" s="15"/>
     </row>
-    <row r="119" spans="1:5" ht="15">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A119" s="13"/>
       <c r="D119" s="15"/>
     </row>
-    <row r="120" spans="1:5" ht="15">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120" s="13"/>
       <c r="D120" s="15"/>
     </row>
-    <row r="121" spans="1:5" ht="15">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D121" s="15"/>
     </row>
-    <row r="122" spans="1:5" ht="15">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122" s="13"/>
     </row>
-    <row r="123" spans="1:5">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123" s="13"/>
       <c r="E123"/>
     </row>
-    <row r="124" spans="1:5" ht="15">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" s="13"/>
     </row>
-    <row r="125" spans="1:5" ht="15">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125" s="13"/>
     </row>
-    <row r="126" spans="1:5" ht="15">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A126" s="13"/>
     </row>
-    <row r="127" spans="1:5" ht="15">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127" s="13"/>
     </row>
-    <row r="128" spans="1:5" ht="15"/>
-    <row r="129" spans="1:5" ht="15">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A129" s="13"/>
       <c r="B129" s="16"/>
       <c r="C129" s="16"/>
       <c r="D129" s="23"/>
       <c r="E129" s="17"/>
     </row>
-    <row r="130" spans="1:5" ht="15">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A130" s="13"/>
       <c r="B130" s="16"/>
       <c r="C130" s="16"/>
       <c r="D130" s="23"/>
       <c r="E130" s="17"/>
     </row>
-    <row r="131" spans="1:5">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131" s="13"/>
       <c r="B131" s="16"/>
       <c r="C131" s="16"/>
       <c r="D131" s="23"/>
       <c r="E131" s="16"/>
     </row>
-    <row r="132" spans="1:5" ht="15">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132" s="13"/>
       <c r="B132" s="16"/>
       <c r="C132" s="16"/>
       <c r="D132" s="23"/>
       <c r="E132" s="17"/>
     </row>
-    <row r="133" spans="1:5" ht="15">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133" s="13"/>
       <c r="B133" s="16"/>
       <c r="C133" s="16"/>
       <c r="D133" s="23"/>
       <c r="E133" s="17"/>
     </row>
-    <row r="134" spans="1:5" ht="15">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134" s="13"/>
       <c r="B134" s="16"/>
       <c r="C134" s="16"/>
       <c r="D134" s="23"/>
       <c r="E134" s="17"/>
     </row>
-    <row r="135" spans="1:5" ht="15"/>
-    <row r="136" spans="1:5" ht="15">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A136" s="13"/>
     </row>
-    <row r="137" spans="1:5" ht="15">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A137" s="13"/>
     </row>
-    <row r="138" spans="1:5" ht="15">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A138" s="13"/>
     </row>
-    <row r="139" spans="1:5" ht="15">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A139" s="13"/>
     </row>
-    <row r="140" spans="1:5" ht="15">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A140" s="13"/>
     </row>
-    <row r="141" spans="1:5" ht="15">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A141" s="13"/>
     </row>
-    <row r="142" spans="1:5" ht="15"/>
-    <row r="143" spans="1:5">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A143" s="13"/>
       <c r="B143" s="16"/>
       <c r="E143" s="21"/>
     </row>
-    <row r="144" spans="1:5">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A144" s="13"/>
       <c r="B144" s="16"/>
       <c r="E144" s="21"/>
     </row>
-    <row r="145" spans="1:5">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A145" s="13"/>
       <c r="B145" s="16"/>
       <c r="E145" s="21"/>
     </row>
-    <row r="146" spans="1:5">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A146" s="13"/>
       <c r="B146" s="16"/>
       <c r="E146" s="22"/>
     </row>
-    <row r="147" spans="1:5">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A147" s="13"/>
       <c r="B147" s="16"/>
       <c r="E147" s="21"/>
     </row>
-    <row r="148" spans="1:5">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A148" s="13"/>
       <c r="B148" s="16"/>
       <c r="E148" s="21"/>
     </row>
-    <row r="149" spans="1:5" ht="15"/>
-    <row r="150" spans="1:5" ht="15">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A150" s="13"/>
       <c r="B150" s="20"/>
       <c r="E150" s="17"/>
     </row>
-    <row r="151" spans="1:5" ht="15">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A151" s="13"/>
       <c r="B151" s="20"/>
       <c r="E151" s="17"/>
     </row>
-    <row r="152" spans="1:5">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A152" s="13"/>
       <c r="B152" s="20"/>
       <c r="E152" s="16"/>
     </row>
-    <row r="153" spans="1:5" ht="15">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153" s="13"/>
       <c r="B153" s="20"/>
       <c r="E153" s="17"/>
     </row>
-    <row r="154" spans="1:5" ht="15">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154" s="13"/>
       <c r="B154" s="20"/>
       <c r="E154" s="17"/>
     </row>
-    <row r="155" spans="1:5" ht="15">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155" s="13"/>
       <c r="E155" s="17"/>
     </row>
-    <row r="156" spans="1:5" ht="15"/>
-    <row r="157" spans="1:5" ht="15">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A157" s="13"/>
     </row>
-    <row r="158" spans="1:5" ht="15">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A158" s="13"/>
     </row>
-    <row r="159" spans="1:5" ht="15">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A159" s="13"/>
     </row>
-    <row r="160" spans="1:5" ht="15">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A160" s="13"/>
     </row>
-    <row r="161" spans="1:2" ht="15">
+    <row r="161" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A161" s="13"/>
     </row>
-    <row r="162" spans="1:2" ht="15">
+    <row r="162" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A162" s="13"/>
     </row>
-    <row r="163" spans="1:2" ht="15">
+    <row r="163" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A163" s="13"/>
     </row>
-    <row r="164" spans="1:2" ht="15">
+    <row r="164" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A164" s="13"/>
     </row>
-    <row r="165" spans="1:2" ht="15">
+    <row r="165" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A165" s="13"/>
     </row>
-    <row r="166" spans="1:2" ht="15">
+    <row r="166" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A166" s="13"/>
     </row>
-    <row r="167" spans="1:2" ht="15">
+    <row r="167" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A167" s="13"/>
     </row>
-    <row r="168" spans="1:2" ht="15">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A168" s="13"/>
     </row>
-    <row r="169" spans="1:2" ht="15">
+    <row r="169" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A169" s="13"/>
     </row>
-    <row r="170" spans="1:2" ht="15">
+    <row r="170" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A170" s="13"/>
     </row>
-    <row r="171" spans="1:2" ht="15">
+    <row r="171" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A171" s="13"/>
     </row>
-    <row r="172" spans="1:2" ht="15">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A172" s="13"/>
     </row>
-    <row r="173" spans="1:2" ht="15">
+    <row r="173" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A173" s="13"/>
     </row>
-    <row r="174" spans="1:2" ht="15">
+    <row r="174" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A174" s="13"/>
       <c r="B174" s="20"/>
     </row>
-    <row r="175" spans="1:2" ht="15">
+    <row r="175" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A175" s="13"/>
       <c r="B175" s="20"/>
     </row>
-    <row r="176" spans="1:2" ht="15">
+    <row r="176" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A176" s="13"/>
     </row>
-    <row r="177" spans="1:1">
+    <row r="177" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A177" s="20"/>
     </row>
   </sheetData>
@@ -1279,19 +1345,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0542F39-F0FF-42BC-8522-46D8537566B3}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A37478F0D103C418E1983367D0E3B29" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0e52e73692c282c4b11ce339126e795d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1a01afa4-83d8-4578-8116-1fe20cdd06b6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d364ad524074f3044f8606d9c9b001a2" ns2:_="">
     <xsd:import namespace="1a01afa4-83d8-4578-8116-1fe20cdd06b6"/>
@@ -1429,6 +1489,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1439,13 +1505,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57E2D867-194E-458C-A857-FF5EE3277888}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC89AADA-5F80-4891-A851-84363269EAD3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1a01afa4-83d8-4578-8116-1fe20cdd06b6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC89AADA-5F80-4891-A851-84363269EAD3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57E2D867-194E-458C-A857-FF5EE3277888}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D5DBCEA-0785-438C-AB6D-531696C8FF28}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D5DBCEA-0785-438C-AB6D-531696C8FF28}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>